<commit_message>
v2.9: fix - 2026/07/20
</commit_message>
<xml_diff>
--- a/resources/M626/spc_sheet_oos_decoration.xlsx
+++ b/resources/M626/spc_sheet_oos_decoration.xlsx
@@ -908,7 +908,7 @@
         <v>-6.5991</v>
       </c>
       <c r="I4">
-        <v>0.05827456140350878</v>
+        <v>0.05827456140350877</v>
       </c>
       <c r="J4">
         <v>6.5</v>
@@ -1482,7 +1482,7 @@
         <v>-7.5721</v>
       </c>
       <c r="I18">
-        <v>-0.4302929824561403</v>
+        <v>-0.4302929824561404</v>
       </c>
       <c r="J18">
         <v>6.5</v>
@@ -1646,7 +1646,7 @@
         <v>-7.3274</v>
       </c>
       <c r="I22">
-        <v>0.0279557522123894</v>
+        <v>0.02795575221238939</v>
       </c>
       <c r="J22">
         <v>6.5</v>
@@ -1728,7 +1728,7 @@
         <v>-6.7783</v>
       </c>
       <c r="I24">
-        <v>-0.0127798245614035</v>
+        <v>-0.01277982456140348</v>
       </c>
       <c r="J24">
         <v>6.5</v>
@@ -1769,7 +1769,7 @@
         <v>-6.7699</v>
       </c>
       <c r="I25">
-        <v>-0.3602491228070176</v>
+        <v>-0.3602491228070175</v>
       </c>
       <c r="J25">
         <v>6.5</v>
@@ -2712,7 +2712,7 @@
         <v>-6.5406</v>
       </c>
       <c r="I48">
-        <v>-0.03138157894736843</v>
+        <v>-0.03138157894736842</v>
       </c>
       <c r="J48">
         <v>6.5</v>
@@ -3655,7 +3655,7 @@
         <v>-7.298</v>
       </c>
       <c r="I71">
-        <v>-0.8348867256637167</v>
+        <v>-0.8348867256637169</v>
       </c>
       <c r="J71">
         <v>6.5</v>
@@ -3778,7 +3778,7 @@
         <v>-4.1674</v>
       </c>
       <c r="I74">
-        <v>0.0329901785714286</v>
+        <v>0.03299017857142858</v>
       </c>
       <c r="J74">
         <v>6.5</v>
@@ -3860,7 +3860,7 @@
         <v>-5.7741</v>
       </c>
       <c r="I76">
-        <v>-0.4322649122807017</v>
+        <v>-0.4322649122807018</v>
       </c>
       <c r="J76">
         <v>6.5</v>
@@ -5172,7 +5172,7 @@
         <v>-13.3146</v>
       </c>
       <c r="I108">
-        <v>0.9303447368421053</v>
+        <v>0.9303447368421052</v>
       </c>
       <c r="J108">
         <v>6.5</v>
@@ -5336,7 +5336,7 @@
         <v>-6.6968</v>
       </c>
       <c r="I112">
-        <v>-0.2789184210526315</v>
+        <v>-0.2789184210526316</v>
       </c>
       <c r="J112">
         <v>6.5</v>
@@ -6197,7 +6197,7 @@
         <v>-6.5323</v>
       </c>
       <c r="I133">
-        <v>-0.7958245614035087</v>
+        <v>-0.7958245614035088</v>
       </c>
       <c r="J133">
         <v>6.5</v>
@@ -6607,7 +6607,7 @@
         <v>-4.8043</v>
       </c>
       <c r="I143">
-        <v>0.3505271929824562</v>
+        <v>0.3505271929824561</v>
       </c>
       <c r="J143">
         <v>6.5</v>
@@ -6853,7 +6853,7 @@
         <v>-10.0195</v>
       </c>
       <c r="I149">
-        <v>0.03782368421052629</v>
+        <v>0.03782368421052633</v>
       </c>
       <c r="J149">
         <v>6.5</v>
@@ -7837,7 +7837,7 @@
         <v>-5.2124</v>
       </c>
       <c r="I173">
-        <v>0.5393429824561404</v>
+        <v>0.5393429824561403</v>
       </c>
       <c r="J173">
         <v>6.5</v>
@@ -7878,7 +7878,7 @@
         <v>-3.8887</v>
       </c>
       <c r="I174">
-        <v>-0.09209473684210528</v>
+        <v>-0.09209473684210527</v>
       </c>
       <c r="J174">
         <v>6.5</v>
@@ -8247,7 +8247,7 @@
         <v>-4.5379</v>
       </c>
       <c r="I183">
-        <v>0.8886482456140352</v>
+        <v>0.888648245614035</v>
       </c>
       <c r="J183">
         <v>6.5</v>
@@ -8370,7 +8370,7 @@
         <v>-1.9388</v>
       </c>
       <c r="I186">
-        <v>2.021550877192983</v>
+        <v>2.021550877192982</v>
       </c>
       <c r="J186">
         <v>6.5</v>

</xml_diff>